<commit_message>
A10 analysis: fix summary wording
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HsFNnGJRzg6EEfnut1VvMX
</commit_message>
<xml_diff>
--- a/loss-time/outputs/Phan_tich_A10.xlsx
+++ b/loss-time/outputs/Phan_tich_A10.xlsx
@@ -812,7 +812,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>8 dòng cả ngày, 2 dòng trùng. Đã tách ra phân tích riêng</t>
+          <t>8 dòng máy dừng cả ngày (1 dòng trong đó cũng là dòng trùng) và 1 dòng trùng khác. Đã tách ra phân tích riêng</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>1. A10 nhỏ về tổng nhưng bị nhiễu: hai nhóm dòng "máy hỏng cả ngày" (CNCR14 tháng 9, CNCR20 ngày 4/4, CNCR01 ngày 4/4) chiếm 479 giờ công, gần 1/3 tổng A10 ghi nhận. Nếu giữ nguyên thì tháng 9 bị thổi phồng (394 giờ thay vì 53 giờ).</t>
+          <t>1. A10 nhỏ về tổng nhưng bị nhiễu: hai nhóm dòng "máy hỏng cả ngày" (CNCR14 tháng 9, CNCR20 ngày 4/4, CNCR01 ngày 4/4) chiếm khoảng 485 giờ công, 35% tổng A10 ghi nhận. Nếu giữ nguyên thì tháng 9 bị thổi phồng (394 giờ thay vì 53 giờ).</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
     <row r="20" ht="34" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>5. 38% dòng chỉ ghi chung chung ("máy hư", "không hoạt động") nên không biết nguyên nhân gốc. Nên yêu cầu bảo trì ghi hiện tượng cụ thể.</t>
+          <t>5. 37% dòng chỉ ghi chung chung ("máy hư", "không hoạt động") nên không biết nguyên nhân gốc. Nên yêu cầu bảo trì ghi hiện tượng cụ thể.</t>
         </is>
       </c>
     </row>
@@ -16604,7 +16604,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Phân loại gần đúng bằng từ khóa. 38% dòng chỉ ghi chung chung nên chưa biết nguyên nhân.</t>
+          <t>Phân loại gần đúng bằng từ khóa. 37% dòng chỉ ghi chung chung nên chưa biết nguyên nhân.</t>
         </is>
       </c>
     </row>

</xml_diff>